<commit_message>
5225 locust test & report
</commit_message>
<xml_diff>
--- a/5225_Project/Ass_1/CloudEco_Project/locust_test.xlsx
+++ b/5225_Project/Ass_1/CloudEco_Project/locust_test.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="17440" windowHeight="13160"/>
+    <workbookView windowWidth="22460" windowHeight="13660" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="17">
   <si>
     <t>1 pod</t>
   </si>
@@ -42,6 +43,42 @@
   </si>
   <si>
     <t>RPS</t>
+  </si>
+  <si>
+    <t>Failure</t>
+  </si>
+  <si>
+    <t>5min/user+1</t>
+  </si>
+  <si>
+    <t>（1 time high response time 6800)</t>
+  </si>
+  <si>
+    <t>(12000,13000,3.1)</t>
+  </si>
+  <si>
+    <t>(16000,18000,3)</t>
+  </si>
+  <si>
+    <t>(20000,76000,6)</t>
+  </si>
+  <si>
+    <t>2 pod</t>
+  </si>
+  <si>
+    <t>2min/user+5</t>
+  </si>
+  <si>
+    <t>4 pod</t>
+  </si>
+  <si>
+    <t>8 pod</t>
+  </si>
+  <si>
+    <t>pods</t>
+  </si>
+  <si>
+    <t>max_users</t>
   </si>
 </sst>
 </file>
@@ -215,12 +252,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -541,7 +584,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -565,16 +608,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -583,90 +626,96 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -947,6 +996,1862 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>Pods vs Maximum Acceptable Users</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet2!$B$1:$E$1</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$E$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>95</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="761566656"/>
+        <c:axId val="465899394"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="761566656"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr defTabSz="914400">
+                  <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t>pod</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:t>s number</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" altLang="zh-CN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="465899394"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="0"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="465899394"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="90200"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr defTabSz="914400">
+                  <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t>max acceptable users</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="761566656"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr lang="zh-CN"/>
+      </a:pPr>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr defTabSz="914400">
+              <a:defRPr lang="zh-CN" sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="75000"/>
+                    <a:lumOff val="25000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>Pods vs Throughput (RPS)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet2!$B$6:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$7:$E$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>5.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12.8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>22.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>32.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="668531791"/>
+        <c:axId val="625074687"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="668531791"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr defTabSz="914400">
+                  <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:t>pods number</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US" altLang="zh-CN"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="625074687"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="625074687"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="lt1">
+                  <a:lumMod val="90200"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr defTabSz="914400">
+                  <a:defRPr lang="zh-CN" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:t>t</a:t>
+                </a:r>
+                <a:r>
+                  <a:t>hroughput (RPS)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="zh-CN" sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="668531791"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr lang="zh-CN"/>
+      </a:pPr>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="10028">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+      <a:effectLst/>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="90200"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="10028">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+      <a:effectLst/>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="lt1">
+            <a:lumMod val="90200"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="1" kern="1200" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>169545</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>118745</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="图表 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5099685" y="445770"/>
+        <a:ext cx="4826000" cy="2875280"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>172085</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>109220</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>121285</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>210820</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="图表 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5102225" y="3522980"/>
+        <a:ext cx="4826000" cy="2875280"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
   <a:themeElements>
@@ -1197,16 +3102,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="3" outlineLevelCol="4"/>
+  <dimension ref="A1:F79"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="11.8557692307692" customWidth="1"/>
     <col min="3" max="3" width="16.0192307692308" customWidth="1"/>
     <col min="4" max="4" width="16.6826923076923" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1221,8 +3126,14 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
       <c r="B2">
         <v>1</v>
       </c>
@@ -1236,7 +3147,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="B3">
         <v>2</v>
       </c>
@@ -1247,16 +3158,1114 @@
         <v>430</v>
       </c>
       <c r="E3">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="B4">
         <v>3</v>
+      </c>
+      <c r="C4">
+        <v>530</v>
+      </c>
+      <c r="D4">
+        <v>620</v>
+      </c>
+      <c r="E4">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>730</v>
+      </c>
+      <c r="D5">
+        <v>820</v>
+      </c>
+      <c r="E5">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>930</v>
+      </c>
+      <c r="D6">
+        <v>1000</v>
+      </c>
+      <c r="E6">
+        <v>5.7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>1000</v>
+      </c>
+      <c r="D7">
+        <v>1100</v>
+      </c>
+      <c r="E7">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>1200</v>
+      </c>
+      <c r="D8">
+        <v>1300</v>
+      </c>
+      <c r="E8">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>1400</v>
+      </c>
+      <c r="D9">
+        <v>1500</v>
+      </c>
+      <c r="E9">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>1500</v>
+      </c>
+      <c r="D10">
+        <v>1600</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>1700</v>
+      </c>
+      <c r="D11">
+        <v>1800</v>
+      </c>
+      <c r="E11">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>1800</v>
+      </c>
+      <c r="D12">
+        <v>1900</v>
+      </c>
+      <c r="E12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <v>2000</v>
+      </c>
+      <c r="D13">
+        <v>2100</v>
+      </c>
+      <c r="E13">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14">
+        <v>2200</v>
+      </c>
+      <c r="D14">
+        <v>2300</v>
+      </c>
+      <c r="E14">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15">
+        <v>2400</v>
+      </c>
+      <c r="D15">
+        <v>2500</v>
+      </c>
+      <c r="E15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16">
+        <v>2500</v>
+      </c>
+      <c r="D16">
+        <v>2600</v>
+      </c>
+      <c r="E16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:6">
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>2600</v>
+      </c>
+      <c r="D17">
+        <v>2700</v>
+      </c>
+      <c r="E17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" s="1" customFormat="1" spans="2:6">
+      <c r="B18" s="1">
+        <v>17</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2900</v>
+      </c>
+      <c r="D18" s="1">
+        <v>3000</v>
+      </c>
+      <c r="E18" s="1">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6">
+      <c r="B19">
+        <v>20</v>
+      </c>
+      <c r="C19">
+        <v>3400</v>
+      </c>
+      <c r="D19">
+        <v>3500</v>
+      </c>
+      <c r="E19">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="20" spans="2:6">
+      <c r="B20">
+        <v>25</v>
+      </c>
+      <c r="C20">
+        <v>4300</v>
+      </c>
+      <c r="D20">
+        <v>4500</v>
+      </c>
+      <c r="E20">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="21" spans="2:6">
+      <c r="B21">
+        <v>30</v>
+      </c>
+      <c r="C21">
+        <v>5000</v>
+      </c>
+      <c r="D21">
+        <v>5100</v>
+      </c>
+      <c r="E21">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="22" spans="2:6">
+      <c r="B22">
+        <v>35</v>
+      </c>
+      <c r="C22">
+        <v>6000</v>
+      </c>
+      <c r="D22">
+        <v>6200</v>
+      </c>
+      <c r="E22">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="23" spans="2:6">
+      <c r="B23">
+        <v>40</v>
+      </c>
+      <c r="C23">
+        <v>6600</v>
+      </c>
+      <c r="D23">
+        <v>6800</v>
+      </c>
+      <c r="E23">
+        <v>5.8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="2:6">
+      <c r="B24">
+        <v>45</v>
+      </c>
+      <c r="C24">
+        <v>7600</v>
+      </c>
+      <c r="D24">
+        <v>7800</v>
+      </c>
+      <c r="E24">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="25" spans="2:6">
+      <c r="B25">
+        <v>50</v>
+      </c>
+      <c r="C25">
+        <v>8400</v>
+      </c>
+      <c r="D25">
+        <v>8700</v>
+      </c>
+      <c r="E25">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:6">
+      <c r="B26">
+        <v>55</v>
+      </c>
+      <c r="C26">
+        <v>9100</v>
+      </c>
+      <c r="D26">
+        <v>9300</v>
+      </c>
+      <c r="E26">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="27" spans="2:6">
+      <c r="B27">
+        <v>60</v>
+      </c>
+      <c r="C27">
+        <v>10000</v>
+      </c>
+      <c r="D27">
+        <v>11000</v>
+      </c>
+      <c r="E27">
+        <v>5.9</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="2:6">
+      <c r="B28">
+        <v>65</v>
+      </c>
+      <c r="C28">
+        <v>11000</v>
+      </c>
+      <c r="D28">
+        <v>12000</v>
+      </c>
+      <c r="E28">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="29" spans="2:6">
+      <c r="B29">
+        <v>70</v>
+      </c>
+      <c r="C29">
+        <v>12000</v>
+      </c>
+      <c r="D29">
+        <v>13000</v>
+      </c>
+      <c r="E29">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="30" spans="2:6">
+      <c r="B30">
+        <v>80</v>
+      </c>
+      <c r="C30">
+        <v>13000</v>
+      </c>
+      <c r="D30">
+        <v>14000</v>
+      </c>
+      <c r="E30">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="31" spans="2:6">
+      <c r="B31">
+        <v>90</v>
+      </c>
+      <c r="C31">
+        <v>15000</v>
+      </c>
+      <c r="D31">
+        <v>16000</v>
+      </c>
+      <c r="E31">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="32" spans="2:6">
+      <c r="B32">
+        <v>100</v>
+      </c>
+      <c r="C32">
+        <v>17000</v>
+      </c>
+      <c r="D32">
+        <v>17000</v>
+      </c>
+      <c r="E32">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="B33">
+        <v>120</v>
+      </c>
+      <c r="C33">
+        <v>20000</v>
+      </c>
+      <c r="D33">
+        <v>21000</v>
+      </c>
+      <c r="E33">
+        <v>5.9</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="B34">
+        <v>140</v>
+      </c>
+      <c r="C34">
+        <v>23000</v>
+      </c>
+      <c r="D34">
+        <v>24000</v>
+      </c>
+      <c r="E34">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="B35">
+        <v>180</v>
+      </c>
+      <c r="C35">
+        <v>30000</v>
+      </c>
+      <c r="D35">
+        <v>31000</v>
+      </c>
+      <c r="E35">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="B36">
+        <v>200</v>
+      </c>
+      <c r="C36">
+        <v>34000</v>
+      </c>
+      <c r="D36">
+        <v>35000</v>
+      </c>
+      <c r="E36">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="B37">
+        <v>240</v>
+      </c>
+      <c r="C37">
+        <v>41000</v>
+      </c>
+      <c r="D37">
+        <v>42000</v>
+      </c>
+      <c r="E37">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="B38">
+        <v>300</v>
+      </c>
+      <c r="C38">
+        <v>51000</v>
+      </c>
+      <c r="D38">
+        <v>52000</v>
+      </c>
+      <c r="E38">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="B39">
+        <v>350</v>
+      </c>
+      <c r="C39">
+        <v>59000</v>
+      </c>
+      <c r="D39">
+        <v>60000</v>
+      </c>
+      <c r="E39">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="B40">
+        <v>400</v>
+      </c>
+      <c r="C40">
+        <v>68000</v>
+      </c>
+      <c r="D40">
+        <v>69000</v>
+      </c>
+      <c r="E40">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="B41">
+        <v>450</v>
+      </c>
+      <c r="C41">
+        <v>76000</v>
+      </c>
+      <c r="D41">
+        <v>77000</v>
+      </c>
+      <c r="E41">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="B42">
+        <v>600</v>
+      </c>
+      <c r="C42">
+        <v>102000</v>
+      </c>
+      <c r="D42">
+        <v>103000</v>
+      </c>
+      <c r="E42">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="B43">
+        <v>1000</v>
+      </c>
+      <c r="C43">
+        <v>137000</v>
+      </c>
+      <c r="D43">
+        <v>138000</v>
+      </c>
+      <c r="E43">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2</v>
+      </c>
+      <c r="D46" t="s">
+        <v>3</v>
+      </c>
+      <c r="E46" t="s">
+        <v>4</v>
+      </c>
+      <c r="F46" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" t="s">
+        <v>12</v>
+      </c>
+      <c r="B47">
+        <v>5</v>
+      </c>
+      <c r="C47">
+        <v>340</v>
+      </c>
+      <c r="D47">
+        <v>550</v>
+      </c>
+      <c r="E47">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="B48">
+        <v>10</v>
+      </c>
+      <c r="C48">
+        <v>780</v>
+      </c>
+      <c r="D48">
+        <v>870</v>
+      </c>
+      <c r="E48">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="B49">
+        <v>15</v>
+      </c>
+      <c r="C49">
+        <v>1000</v>
+      </c>
+      <c r="D49">
+        <v>1400</v>
+      </c>
+      <c r="E49">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="B50">
+        <v>20</v>
+      </c>
+      <c r="C50">
+        <v>1500</v>
+      </c>
+      <c r="D50">
+        <v>1700</v>
+      </c>
+      <c r="E50">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="B51">
+        <v>25</v>
+      </c>
+      <c r="C51">
+        <v>1800</v>
+      </c>
+      <c r="D51">
+        <v>2300</v>
+      </c>
+      <c r="E51">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="B52">
+        <v>30</v>
+      </c>
+      <c r="C52">
+        <v>2200</v>
+      </c>
+      <c r="D52">
+        <v>2600</v>
+      </c>
+      <c r="E52">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="53" s="2" customFormat="1" spans="1:6">
+      <c r="B53" s="2">
+        <v>35</v>
+      </c>
+      <c r="C53" s="2">
+        <v>2500</v>
+      </c>
+      <c r="D53" s="2">
+        <v>3100</v>
+      </c>
+      <c r="E53" s="2">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2</v>
+      </c>
+      <c r="D56" t="s">
+        <v>3</v>
+      </c>
+      <c r="E56" t="s">
+        <v>4</v>
+      </c>
+      <c r="F56" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>12</v>
+      </c>
+      <c r="B57">
+        <v>30</v>
+      </c>
+      <c r="C57">
+        <v>1300</v>
+      </c>
+      <c r="D57">
+        <v>1400</v>
+      </c>
+      <c r="E57">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="B58">
+        <v>35</v>
+      </c>
+      <c r="C58">
+        <v>1600</v>
+      </c>
+      <c r="D58">
+        <v>1800</v>
+      </c>
+      <c r="E58">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="B59">
+        <v>40</v>
+      </c>
+      <c r="C59">
+        <v>1800</v>
+      </c>
+      <c r="D59">
+        <v>1900</v>
+      </c>
+      <c r="E59">
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="B60">
+        <v>45</v>
+      </c>
+      <c r="C60">
+        <v>2000</v>
+      </c>
+      <c r="D60">
+        <v>2100</v>
+      </c>
+      <c r="E60">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="B61">
+        <v>50</v>
+      </c>
+      <c r="C61">
+        <v>2200</v>
+      </c>
+      <c r="D61">
+        <v>2400</v>
+      </c>
+      <c r="E61">
+        <v>22.6</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="B62">
+        <v>55</v>
+      </c>
+      <c r="C62">
+        <v>2400</v>
+      </c>
+      <c r="D62">
+        <v>2600</v>
+      </c>
+      <c r="E62">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="B63">
+        <v>60</v>
+      </c>
+      <c r="C63">
+        <v>2600</v>
+      </c>
+      <c r="D63">
+        <v>2800</v>
+      </c>
+      <c r="E63">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="64" s="1" customFormat="1" spans="1:6">
+      <c r="B64" s="1">
+        <v>65</v>
+      </c>
+      <c r="C64" s="1">
+        <v>2900</v>
+      </c>
+      <c r="D64" s="1">
+        <v>3100</v>
+      </c>
+      <c r="E64" s="1">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B67" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>2</v>
+      </c>
+      <c r="D67" t="s">
+        <v>3</v>
+      </c>
+      <c r="E67" t="s">
+        <v>4</v>
+      </c>
+      <c r="F67" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>12</v>
+      </c>
+      <c r="B68">
+        <v>40</v>
+      </c>
+      <c r="C68">
+        <v>1200</v>
+      </c>
+      <c r="D68">
+        <v>1400</v>
+      </c>
+      <c r="E68">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="B69">
+        <v>45</v>
+      </c>
+      <c r="C69">
+        <v>1400</v>
+      </c>
+      <c r="D69">
+        <v>1600</v>
+      </c>
+      <c r="E69">
+        <v>32.7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="B70">
+        <v>50</v>
+      </c>
+      <c r="C70">
+        <v>1500</v>
+      </c>
+      <c r="D70">
+        <v>1700</v>
+      </c>
+      <c r="E70">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="B71">
+        <v>55</v>
+      </c>
+      <c r="C71">
+        <v>1700</v>
+      </c>
+      <c r="D71">
+        <v>1900</v>
+      </c>
+      <c r="E71">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="B72">
+        <v>60</v>
+      </c>
+      <c r="C72">
+        <v>1800</v>
+      </c>
+      <c r="D72">
+        <v>2000</v>
+      </c>
+      <c r="E72">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="B73">
+        <v>65</v>
+      </c>
+      <c r="C73">
+        <v>2000</v>
+      </c>
+      <c r="D73">
+        <v>2100</v>
+      </c>
+      <c r="E73">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="B74">
+        <v>70</v>
+      </c>
+      <c r="C74">
+        <v>2100</v>
+      </c>
+      <c r="D74">
+        <v>2300</v>
+      </c>
+      <c r="E74">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="B75">
+        <v>75</v>
+      </c>
+      <c r="C75">
+        <v>2300</v>
+      </c>
+      <c r="D75">
+        <v>2500</v>
+      </c>
+      <c r="E75">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="B76">
+        <v>80</v>
+      </c>
+      <c r="C76">
+        <v>2400</v>
+      </c>
+      <c r="D76">
+        <v>2600</v>
+      </c>
+      <c r="E76">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="B77">
+        <v>85</v>
+      </c>
+      <c r="C77">
+        <v>2600</v>
+      </c>
+      <c r="D77">
+        <v>2800</v>
+      </c>
+      <c r="E77">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="B78">
+        <v>90</v>
+      </c>
+      <c r="C78">
+        <v>2700</v>
+      </c>
+      <c r="D78">
+        <v>2900</v>
+      </c>
+      <c r="E78">
+        <v>32.9</v>
+      </c>
+    </row>
+    <row r="79" s="1" customFormat="1" spans="1:6">
+      <c r="B79" s="1">
+        <v>95</v>
+      </c>
+      <c r="C79" s="1">
+        <v>2900</v>
+      </c>
+      <c r="D79" s="1">
+        <v>3100</v>
+      </c>
+      <c r="E79" s="1">
+        <v>32.8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="6" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="10.0384615384615" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>4</v>
+      </c>
+      <c r="E1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>17</v>
+      </c>
+      <c r="C2">
+        <v>35</v>
+      </c>
+      <c r="D2">
+        <v>65</v>
+      </c>
+      <c r="E2">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>5.8</v>
+      </c>
+      <c r="C7">
+        <v>12.8</v>
+      </c>
+      <c r="D7">
+        <v>22.7</v>
+      </c>
+      <c r="E7">
+        <v>32.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>